<commit_message>
Finalizando o projeto com as partes das validações
</commit_message>
<xml_diff>
--- a/comparacao_impressoras/comparacoes.xlsx
+++ b/comparacao_impressoras/comparacoes.xlsx
@@ -481,7 +481,11 @@
       <c r="F2" t="n">
         <v>757</v>
       </c>
-      <c r="G2" t="inlineStr"/>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -508,7 +512,11 @@
       <c r="F3" t="n">
         <v>13862</v>
       </c>
-      <c r="G3" t="inlineStr"/>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -535,7 +543,11 @@
       <c r="F4" t="n">
         <v>621</v>
       </c>
-      <c r="G4" t="inlineStr"/>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -562,7 +574,11 @@
       <c r="F5" t="n">
         <v>2478</v>
       </c>
-      <c r="G5" t="inlineStr"/>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -589,7 +605,11 @@
       <c r="F6" t="n">
         <v>759</v>
       </c>
-      <c r="G6" t="inlineStr"/>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -616,7 +636,11 @@
       <c r="F7" t="n">
         <v>3388</v>
       </c>
-      <c r="G7" t="inlineStr"/>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -643,7 +667,11 @@
       <c r="F8" t="n">
         <v>685</v>
       </c>
-      <c r="G8" t="inlineStr"/>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -670,7 +698,11 @@
       <c r="F9" t="n">
         <v>4044</v>
       </c>
-      <c r="G9" t="inlineStr"/>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -728,7 +760,11 @@
       <c r="F11" t="n">
         <v>374</v>
       </c>
-      <c r="G11" t="inlineStr"/>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -755,7 +791,11 @@
       <c r="F12" t="n">
         <v>6577</v>
       </c>
-      <c r="G12" t="inlineStr"/>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -782,7 +822,11 @@
       <c r="F13" t="n">
         <v>828</v>
       </c>
-      <c r="G13" t="inlineStr"/>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -809,7 +853,11 @@
       <c r="F14" t="n">
         <v>1030</v>
       </c>
-      <c r="G14" t="inlineStr"/>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -836,7 +884,11 @@
       <c r="F15" t="n">
         <v>3616</v>
       </c>
-      <c r="G15" t="inlineStr"/>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -863,7 +915,11 @@
       <c r="F16" t="n">
         <v>3042</v>
       </c>
-      <c r="G16" t="inlineStr"/>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -890,7 +946,11 @@
       <c r="F17" t="n">
         <v>1063</v>
       </c>
-      <c r="G17" t="inlineStr"/>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -917,7 +977,11 @@
       <c r="F18" t="n">
         <v>217</v>
       </c>
-      <c r="G18" t="inlineStr"/>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -944,7 +1008,11 @@
       <c r="F19" t="n">
         <v>56</v>
       </c>
-      <c r="G19" t="inlineStr"/>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -971,7 +1039,11 @@
       <c r="F20" t="n">
         <v>613</v>
       </c>
-      <c r="G20" t="inlineStr"/>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -998,7 +1070,11 @@
       <c r="F21" t="n">
         <v>13362</v>
       </c>
-      <c r="G21" t="inlineStr"/>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1025,7 +1101,11 @@
       <c r="F22" t="n">
         <v>1094</v>
       </c>
-      <c r="G22" t="inlineStr"/>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1052,7 +1132,11 @@
       <c r="F23" t="n">
         <v>1242</v>
       </c>
-      <c r="G23" t="inlineStr"/>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1079,7 +1163,11 @@
       <c r="F24" t="n">
         <v>820</v>
       </c>
-      <c r="G24" t="inlineStr"/>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1106,7 +1194,11 @@
       <c r="F25" t="n">
         <v>763</v>
       </c>
-      <c r="G25" t="inlineStr"/>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1133,7 +1225,11 @@
       <c r="F26" t="n">
         <v>1400</v>
       </c>
-      <c r="G26" t="inlineStr"/>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1160,7 +1256,11 @@
       <c r="F27" t="n">
         <v>10672</v>
       </c>
-      <c r="G27" t="inlineStr"/>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1187,7 +1287,11 @@
       <c r="F28" t="n">
         <v>9311</v>
       </c>
-      <c r="G28" t="inlineStr"/>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -1214,7 +1318,11 @@
       <c r="F29" t="n">
         <v>5568</v>
       </c>
-      <c r="G29" t="inlineStr"/>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -1241,7 +1349,11 @@
       <c r="F30" t="n">
         <v>5525</v>
       </c>
-      <c r="G30" t="inlineStr"/>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -1268,7 +1380,11 @@
       <c r="F31" t="n">
         <v>2672</v>
       </c>
-      <c r="G31" t="inlineStr"/>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -1295,7 +1411,11 @@
       <c r="F32" t="n">
         <v>2052</v>
       </c>
-      <c r="G32" t="inlineStr"/>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -1322,7 +1442,11 @@
       <c r="F33" t="n">
         <v>3608</v>
       </c>
-      <c r="G33" t="inlineStr"/>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -1349,7 +1473,11 @@
       <c r="F34" t="n">
         <v>78</v>
       </c>
-      <c r="G34" t="inlineStr"/>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -1845,7 +1973,11 @@
       <c r="F2" t="n">
         <v>757</v>
       </c>
-      <c r="G2" t="inlineStr"/>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1872,7 +2004,11 @@
       <c r="F3" t="n">
         <v>11512</v>
       </c>
-      <c r="G3" t="inlineStr"/>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1899,7 +2035,11 @@
       <c r="F4" t="n">
         <v>623</v>
       </c>
-      <c r="G4" t="inlineStr"/>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1926,7 +2066,11 @@
       <c r="F5" t="n">
         <v>2307</v>
       </c>
-      <c r="G5" t="inlineStr"/>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1953,7 +2097,11 @@
       <c r="F6" t="n">
         <v>773</v>
       </c>
-      <c r="G6" t="inlineStr"/>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1980,7 +2128,11 @@
       <c r="F7" t="n">
         <v>3475</v>
       </c>
-      <c r="G7" t="inlineStr"/>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -2007,7 +2159,11 @@
       <c r="F8" t="n">
         <v>708</v>
       </c>
-      <c r="G8" t="inlineStr"/>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -2034,7 +2190,11 @@
       <c r="F9" t="n">
         <v>2853</v>
       </c>
-      <c r="G9" t="inlineStr"/>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -2084,7 +2244,11 @@
       <c r="F11" t="n">
         <v>387</v>
       </c>
-      <c r="G11" t="inlineStr"/>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -2111,7 +2275,11 @@
       <c r="F12" t="n">
         <v>6524</v>
       </c>
-      <c r="G12" t="inlineStr"/>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -2138,7 +2306,11 @@
       <c r="F13" t="n">
         <v>713</v>
       </c>
-      <c r="G13" t="inlineStr"/>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -2165,7 +2337,11 @@
       <c r="F14" t="n">
         <v>1019</v>
       </c>
-      <c r="G14" t="inlineStr"/>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -2192,7 +2368,11 @@
       <c r="F15" t="n">
         <v>5423</v>
       </c>
-      <c r="G15" t="inlineStr"/>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -2219,7 +2399,11 @@
       <c r="F16" t="n">
         <v>1002</v>
       </c>
-      <c r="G16" t="inlineStr"/>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -2246,7 +2430,11 @@
       <c r="F17" t="n">
         <v>792</v>
       </c>
-      <c r="G17" t="inlineStr"/>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -2273,7 +2461,11 @@
       <c r="F18" t="n">
         <v>167</v>
       </c>
-      <c r="G18" t="inlineStr"/>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -2331,7 +2523,11 @@
       <c r="F20" t="n">
         <v>591</v>
       </c>
-      <c r="G20" t="inlineStr"/>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -2358,7 +2554,11 @@
       <c r="F21" t="n">
         <v>11419</v>
       </c>
-      <c r="G21" t="inlineStr"/>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -2385,7 +2585,11 @@
       <c r="F22" t="n">
         <v>536</v>
       </c>
-      <c r="G22" t="inlineStr"/>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -2412,7 +2616,11 @@
       <c r="F23" t="n">
         <v>39290</v>
       </c>
-      <c r="G23" t="inlineStr"/>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -2439,7 +2647,11 @@
       <c r="F24" t="n">
         <v>1314</v>
       </c>
-      <c r="G24" t="inlineStr"/>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -2466,7 +2678,11 @@
       <c r="F25" t="n">
         <v>867</v>
       </c>
-      <c r="G25" t="inlineStr"/>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -2493,7 +2709,11 @@
       <c r="F26" t="n">
         <v>1279</v>
       </c>
-      <c r="G26" t="inlineStr"/>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -2520,7 +2740,11 @@
       <c r="F27" t="n">
         <v>4893</v>
       </c>
-      <c r="G27" t="inlineStr"/>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -2547,7 +2771,11 @@
       <c r="F28" t="n">
         <v>9310</v>
       </c>
-      <c r="G28" t="inlineStr"/>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -2574,7 +2802,11 @@
       <c r="F29" t="n">
         <v>5172</v>
       </c>
-      <c r="G29" t="inlineStr"/>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -2601,7 +2833,11 @@
       <c r="F30" t="n">
         <v>5252</v>
       </c>
-      <c r="G30" t="inlineStr"/>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -2628,7 +2864,11 @@
       <c r="F31" t="n">
         <v>536</v>
       </c>
-      <c r="G31" t="inlineStr"/>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -2655,7 +2895,11 @@
       <c r="F32" t="n">
         <v>1719</v>
       </c>
-      <c r="G32" t="inlineStr"/>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -2682,7 +2926,11 @@
       <c r="F33" t="n">
         <v>2266</v>
       </c>
-      <c r="G33" t="inlineStr"/>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -2709,7 +2957,11 @@
       <c r="F34" t="n">
         <v>3324</v>
       </c>
-      <c r="G34" t="inlineStr"/>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -2736,7 +2988,11 @@
       <c r="F35" t="n">
         <v>78</v>
       </c>
-      <c r="G35" t="inlineStr"/>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -3240,7 +3496,11 @@
       <c r="F2" t="n">
         <v>1514</v>
       </c>
-      <c r="G2" t="inlineStr"/>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -3267,7 +3527,11 @@
       <c r="F3" t="n">
         <v>24991</v>
       </c>
-      <c r="G3" t="inlineStr"/>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -3294,7 +3558,11 @@
       <c r="F4" t="n">
         <v>8039</v>
       </c>
-      <c r="G4" t="inlineStr"/>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -3321,7 +3589,11 @@
       <c r="F5" t="n">
         <v>4476</v>
       </c>
-      <c r="G5" t="inlineStr"/>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -3348,7 +3620,11 @@
       <c r="F6" t="n">
         <v>1483</v>
       </c>
-      <c r="G6" t="inlineStr"/>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -3375,7 +3651,11 @@
       <c r="F7" t="n">
         <v>8404</v>
       </c>
-      <c r="G7" t="inlineStr"/>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -3402,7 +3682,11 @@
       <c r="F8" t="n">
         <v>5231</v>
       </c>
-      <c r="G8" t="inlineStr"/>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -3429,7 +3713,11 @@
       <c r="F9" t="n">
         <v>6132</v>
       </c>
-      <c r="G9" t="inlineStr"/>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -3456,7 +3744,11 @@
       <c r="F10" t="n">
         <v>662</v>
       </c>
-      <c r="G10" t="inlineStr"/>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -3483,7 +3775,11 @@
       <c r="F11" t="n">
         <v>13108</v>
       </c>
-      <c r="G11" t="inlineStr"/>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -3510,7 +3806,11 @@
       <c r="F12" t="n">
         <v>973</v>
       </c>
-      <c r="G12" t="inlineStr"/>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -3537,7 +3837,11 @@
       <c r="F13" t="n">
         <v>1422</v>
       </c>
-      <c r="G13" t="inlineStr"/>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -3564,7 +3868,11 @@
       <c r="F14" t="n">
         <v>1976</v>
       </c>
-      <c r="G14" t="inlineStr"/>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -3591,7 +3899,11 @@
       <c r="F15" t="n">
         <v>8241</v>
       </c>
-      <c r="G15" t="inlineStr"/>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -3618,7 +3930,11 @@
       <c r="F16" t="n">
         <v>3145</v>
       </c>
-      <c r="G16" t="inlineStr"/>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -3645,7 +3961,11 @@
       <c r="F17" t="n">
         <v>1542</v>
       </c>
-      <c r="G17" t="inlineStr"/>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -3672,7 +3992,11 @@
       <c r="F18" t="n">
         <v>371</v>
       </c>
-      <c r="G18" t="inlineStr"/>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -3699,7 +4023,11 @@
       <c r="F19" t="n">
         <v>71</v>
       </c>
-      <c r="G19" t="inlineStr"/>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -3726,7 +4054,11 @@
       <c r="F20" t="n">
         <v>995</v>
       </c>
-      <c r="G20" t="inlineStr"/>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -3753,7 +4085,11 @@
       <c r="F21" t="n">
         <v>16431</v>
       </c>
-      <c r="G21" t="inlineStr"/>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -3780,7 +4116,11 @@
       <c r="F22" t="n">
         <v>1962</v>
       </c>
-      <c r="G22" t="inlineStr"/>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -3830,7 +4170,11 @@
       <c r="F24" t="n">
         <v>1906</v>
       </c>
-      <c r="G24" t="inlineStr"/>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -3857,7 +4201,11 @@
       <c r="F25" t="n">
         <v>1905</v>
       </c>
-      <c r="G25" t="inlineStr"/>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -3884,7 +4232,11 @@
       <c r="F26" t="n">
         <v>9566</v>
       </c>
-      <c r="G26" t="inlineStr"/>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -3911,7 +4263,11 @@
       <c r="F27" t="n">
         <v>12934</v>
       </c>
-      <c r="G27" t="inlineStr"/>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -3938,7 +4294,11 @@
       <c r="F28" t="n">
         <v>18620</v>
       </c>
-      <c r="G28" t="inlineStr"/>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -3965,7 +4325,11 @@
       <c r="F29" t="n">
         <v>10607</v>
       </c>
-      <c r="G29" t="inlineStr"/>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -3992,7 +4356,11 @@
       <c r="F30" t="n">
         <v>11642</v>
       </c>
-      <c r="G30" t="inlineStr"/>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -4019,7 +4387,11 @@
       <c r="F31" t="n">
         <v>748</v>
       </c>
-      <c r="G31" t="inlineStr"/>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -4046,7 +4418,11 @@
       <c r="F32" t="n">
         <v>4230</v>
       </c>
-      <c r="G32" t="inlineStr"/>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -4096,7 +4472,11 @@
       <c r="F34" t="n">
         <v>4739</v>
       </c>
-      <c r="G34" t="inlineStr"/>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -4123,7 +4503,11 @@
       <c r="F35" t="n">
         <v>156</v>
       </c>
-      <c r="G35" t="inlineStr"/>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -4627,7 +5011,11 @@
       <c r="F2" t="n">
         <v>1514</v>
       </c>
-      <c r="G2" t="inlineStr"/>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -4654,7 +5042,11 @@
       <c r="F3" t="n">
         <v>22622</v>
       </c>
-      <c r="G3" t="inlineStr"/>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -4681,7 +5073,11 @@
       <c r="F4" t="n">
         <v>6529</v>
       </c>
-      <c r="G4" t="inlineStr"/>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -4708,7 +5104,11 @@
       <c r="F5" t="n">
         <v>5003</v>
       </c>
-      <c r="G5" t="inlineStr"/>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -4735,7 +5135,11 @@
       <c r="F6" t="n">
         <v>752</v>
       </c>
-      <c r="G6" t="inlineStr"/>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -4762,7 +5166,11 @@
       <c r="F7" t="n">
         <v>8081</v>
       </c>
-      <c r="G7" t="inlineStr"/>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -4789,7 +5197,11 @@
       <c r="F8" t="n">
         <v>4384</v>
       </c>
-      <c r="G8" t="inlineStr"/>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -4816,7 +5228,11 @@
       <c r="F9" t="n">
         <v>8711</v>
       </c>
-      <c r="G9" t="inlineStr"/>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -4843,7 +5259,11 @@
       <c r="F10" t="n">
         <v>71419</v>
       </c>
-      <c r="G10" t="inlineStr"/>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -4870,7 +5290,11 @@
       <c r="F11" t="n">
         <v>13095</v>
       </c>
-      <c r="G11" t="inlineStr"/>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -4897,7 +5321,11 @@
       <c r="F12" t="n">
         <v>920</v>
       </c>
-      <c r="G12" t="inlineStr"/>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -4924,7 +5352,11 @@
       <c r="F13" t="n">
         <v>863</v>
       </c>
-      <c r="G13" t="inlineStr"/>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -4951,7 +5383,11 @@
       <c r="F14" t="n">
         <v>1989</v>
       </c>
-      <c r="G14" t="inlineStr"/>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -4978,7 +5414,11 @@
       <c r="F15" t="n">
         <v>4574</v>
       </c>
-      <c r="G15" t="inlineStr"/>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -5028,7 +5468,11 @@
       <c r="F17" t="n">
         <v>6932</v>
       </c>
-      <c r="G17" t="inlineStr"/>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -5086,7 +5530,11 @@
       <c r="F19" t="n">
         <v>3855</v>
       </c>
-      <c r="G19" t="inlineStr"/>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -5113,7 +5561,11 @@
       <c r="F20" t="n">
         <v>616</v>
       </c>
-      <c r="G20" t="inlineStr"/>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -5140,7 +5592,11 @@
       <c r="F21" t="n">
         <v>25729</v>
       </c>
-      <c r="G21" t="inlineStr"/>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -5167,7 +5623,11 @@
       <c r="F22" t="n">
         <v>8070</v>
       </c>
-      <c r="G22" t="inlineStr"/>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -5194,7 +5654,11 @@
       <c r="F23" t="n">
         <v>1832</v>
       </c>
-      <c r="G23" t="inlineStr"/>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -5221,7 +5685,11 @@
       <c r="F24" t="n">
         <v>1867</v>
       </c>
-      <c r="G24" t="inlineStr"/>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -5248,7 +5716,11 @@
       <c r="F25" t="n">
         <v>8009</v>
       </c>
-      <c r="G25" t="inlineStr"/>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -5275,7 +5747,11 @@
       <c r="F26" t="n">
         <v>25726</v>
       </c>
-      <c r="G26" t="inlineStr"/>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -5302,7 +5778,11 @@
       <c r="F27" t="n">
         <v>18620</v>
       </c>
-      <c r="G27" t="inlineStr"/>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -5329,7 +5809,11 @@
       <c r="F28" t="n">
         <v>10549</v>
       </c>
-      <c r="G28" t="inlineStr"/>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -5356,7 +5840,11 @@
       <c r="F29" t="n">
         <v>15886</v>
       </c>
-      <c r="G29" t="inlineStr"/>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -5383,7 +5871,11 @@
       <c r="F30" t="n">
         <v>820</v>
       </c>
-      <c r="G30" t="inlineStr"/>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -5410,7 +5902,11 @@
       <c r="F31" t="n">
         <v>4054</v>
       </c>
-      <c r="G31" t="inlineStr"/>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -5437,7 +5933,11 @@
       <c r="F32" t="n">
         <v>3625</v>
       </c>
-      <c r="G32" t="inlineStr"/>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -5464,7 +5964,11 @@
       <c r="F33" t="n">
         <v>156</v>
       </c>
-      <c r="G33" t="inlineStr"/>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">

</xml_diff>